<commit_message>
Family Average script added
</commit_message>
<xml_diff>
--- a/tests/input_file/input_file.xlsx
+++ b/tests/input_file/input_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Arash_repo\load-arena\tests\input_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D64E7A-A042-48C6-A859-D77EF1732A50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE078653-EEAF-47DC-A55E-65AC0B7A554E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-118" yWindow="-118" windowWidth="25370" windowHeight="13759" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="759" yWindow="759" windowWidth="18851" windowHeight="9845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Timeseries config" sheetId="2" r:id="rId1"/>
@@ -40,9 +40,6 @@
     <t>mean</t>
   </si>
   <si>
-    <t>DLC12</t>
-  </si>
-  <si>
     <t>dlc12_wsp04_wdir000_s023004</t>
   </si>
   <si>
@@ -53,6 +50,9 @@
   </si>
   <si>
     <t>dlc12_wsp12_wdir000_s038012</t>
+  </si>
+  <si>
+    <t>d:\Arash_repo\load-arena\tests\h2_res\dlc12\</t>
   </si>
 </sst>
 </file>
@@ -424,7 +424,7 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="1" max="1" width="38.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
     <col min="4" max="4" width="5" customWidth="1"/>
@@ -450,10 +450,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -467,10 +467,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -484,10 +484,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -501,10 +501,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>2</v>

</xml_diff>